<commit_message>
Clean up exhibitor workbook after independent verification
- Strip an invisible right-to-left mark copied from the site
  ("QURTOBA FOR EXPORT") and normalize a non-breaking space, so exact
  lookups and "begins with" filters work in Excel.
- Spell "United States Of America" the way the site's own country filter
  does; the summary now counts 44 countries, matching the site.
- Add notes for the "Hal l2" stand typo, the tag the site itself cuts off
  at 240 characters, and what "Not stated" covers in the hall table.
- Use one link font throughout, make the source URL clickable, and stamp
  the snapshot time, since the site's list is still changing.
- Rebuilt from the live page: still 573 exhibitors on 29 pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CmU22w65Cq7PJsk63QCTRt
</commit_message>
<xml_diff>
--- a/foodafrica-exhibitors/FoodAfrica_2026_Exhibitors.xlsx
+++ b/foodafrica-exhibitors/FoodAfrica_2026_Exhibitors.xlsx
@@ -27,11 +27,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="10"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
     <font>
       <b val="1"/>
@@ -67,11 +64,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -82,18 +78,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -2279,7 +2277,11 @@
       <c r="J45" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K45" s="3" t="inlineStr"/>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>A tag on this row stops at 240 characters on the site itself (cut off there).</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -5200,7 +5202,11 @@
       <c r="J118" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="K118" s="3" t="inlineStr"/>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>Hall read from the site's stand text 'Hal l2/ F71'.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -19044,7 +19050,7 @@
       </c>
       <c r="B459" s="3" t="inlineStr">
         <is>
-          <t>‏QURTOBA FOR EXPORT</t>
+          <t>QURTOBA FOR EXPORT</t>
         </is>
       </c>
       <c r="C459" s="2" t="inlineStr">
@@ -22531,7 +22537,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>United States Of America</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -22567,7 +22573,11 @@
       <c r="J545" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K545" s="3" t="inlineStr"/>
+      <c r="K545" s="3" t="inlineStr">
+        <is>
+          <t>Country written 'United States Of America' on this row of the site; shown as spelled in the site's country filter.</t>
+        </is>
+      </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="n">
@@ -23421,12 +23431,12 @@
       </c>
       <c r="G567" s="3" t="inlineStr">
         <is>
-          <t>Beverages; Dairy-Free Products; Edible Oils; Gluten-Free Products; Halal Products; Herbs &amp; Spices; Milk, Cheese &amp; Dairy Products; Private Label Products; Special Diet &amp; Functional Food; Tea, Coffee &amp; Herbal Infusions; Coconut cream powder; Ginger powder; Non-dairy creamer; Palm Kernel Fatty Acid Distillate; Refined Bleached Deodorized Palm Kernel Oil; Whipping cream &amp; Cream cheese powder</t>
+          <t>Beverages; Dairy-Free Products; Edible Oils; Gluten-Free Products; Halal Products; Herbs &amp; Spices; Milk, Cheese &amp; Dairy Products; Private Label Products; Special Diet &amp; Functional Food; Tea, Coffee &amp; Herbal Infusions</t>
         </is>
       </c>
       <c r="H567" s="3" t="inlineStr">
         <is>
-          <t>Food Products; Specialty Products; Coconut cream powder; Ginger powder; Non-dairy creamer; Palm Kernel Fatty Acid Distillate; Refined Bleached Deodorized Palm Kernel Oil; Whipping cream &amp; Cream cheese powder</t>
+          <t>Food Products; Specialty Products</t>
         </is>
       </c>
       <c r="I567" s="4" t="inlineStr">
@@ -23954,7 +23964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -23984,12 +23994,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Extracted on</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
+          <t>Snapshot taken</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28 05:02 UTC</t>
         </is>
       </c>
     </row>
@@ -23999,7 +24009,7 @@
           <t>Total exhibitors</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>573</v>
       </c>
     </row>
@@ -24009,8 +24019,8 @@
           <t>Countries</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>45</v>
+      <c r="B6" s="8" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="7">
@@ -24019,7 +24029,7 @@
           <t>Pages on site (20 per page)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>29</v>
       </c>
     </row>
@@ -24029,7 +24039,7 @@
           <t>With profiles / categories</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>210</v>
       </c>
     </row>
@@ -24039,7 +24049,7 @@
           <t>With logo</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>220</v>
       </c>
     </row>
@@ -24053,249 +24063,243 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Rows are in the site's own A–Z order; 'Page on Site' is the list page each exhibitor appears on.</t>
+          <t>The site's list is live: exhibitors can still be added or edited before the show, so this is a snapshot as of the time above.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>'Hall' and 'Stand No.' are split out of the site's stand text, which is kept unchanged in 'Stand (as listed on site)'. A stand shown as '-' on the site is left blank in 'Stand No.'.</t>
+          <t>Rows are in the site's own A–Z order; 'Page on Site' is the list page each exhibitor appears on.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Profiles and Categories are the tags each exhibitor selected (some are free text), separated by '; '.</t>
+          <t>'Hall' and 'Stand No.' are split out of the site's stand text, which is kept unchanged in 'Stand (as listed on site)'. A stand shown as '-' on the site is left blank in 'Stand No.'.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Profiles and Categories are the tags each exhibitor selected (some are free text), separated by '; '.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>The list page's heading says it covers Halls 2–6.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>'Not stated' in the hall table covers 40 exhibitors listed with a stand code but no hall, and 3 with no stand listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Hall</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Exhibitors</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Hall 2</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Hall 3</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>135</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hall 4</t>
+          <t>Hall 2</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hall 5</t>
+          <t>Hall 3</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hall 6</t>
+          <t>Hall 4</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>35</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Hall 5</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hall 6</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B25" t="n">
         <v>43</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Exhibitors</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Türkiye</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>33</v>
+        <v>332</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Guinea</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Guinea</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -24305,27 +24309,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Azerbaijan</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -24335,7 +24339,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -24345,7 +24349,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Macedonia</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -24355,7 +24359,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -24365,7 +24369,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sudan</t>
+          <t>Macedonia</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -24375,7 +24379,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -24385,7 +24389,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Syria</t>
+          <t>Sudan</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -24395,7 +24399,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -24405,37 +24409,37 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Syria</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -24445,7 +24449,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -24455,7 +24459,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>England</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -24465,7 +24469,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -24475,7 +24479,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -24485,7 +24489,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -24495,7 +24499,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Madagascar</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -24505,7 +24509,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -24515,7 +24519,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -24525,7 +24529,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Palestine</t>
+          <t>Madagascar</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -24535,7 +24539,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -24545,7 +24549,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -24555,7 +24559,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Palestine</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -24565,7 +24569,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -24575,7 +24579,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -24585,7 +24589,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -24595,7 +24599,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>United States Of America</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -24605,20 +24609,35 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A16:C16"/>
     <mergeCell ref="A15:C15"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>